<commit_message>
security: remove hardcoded service_role key, hash passwords, restrict CORS
</commit_message>
<xml_diff>
--- a/KalkulatorPosisiKas.xlsx
+++ b/KalkulatorPosisiKas.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29127"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Project\KasM\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Project\KasM\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{3265D5E4-22D3-4D33-9025-C4DD9721035D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3384BD9C-628C-4D5E-ACFC-262F06544DE3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="7590" yWindow="2025" windowWidth="15180" windowHeight="9210" xr2:uid="{39C8A8B0-5FB8-4A23-A659-AD09C2EB872F}"/>
+    <workbookView xWindow="1540" yWindow="810" windowWidth="12620" windowHeight="8500" xr2:uid="{39C8A8B0-5FB8-4A23-A659-AD09C2EB872F}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet2" sheetId="1" r:id="rId1"/>
@@ -20,12 +20,21 @@
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
     </ext>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="26" uniqueCount="23">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="26" uniqueCount="24">
   <si>
     <t>Contoh</t>
   </si>
@@ -57,9 +66,6 @@
     <t>Penerimaan</t>
   </si>
   <si>
-    <t>Antar Teller</t>
-  </si>
-  <si>
     <t>Pembayaran</t>
   </si>
   <si>
@@ -72,9 +78,6 @@
     <t>Setor Sore</t>
   </si>
   <si>
-    <t>Estim Kredit - (Bon Pagi+Bon Tambahan)+Setor Tambahan</t>
-  </si>
-  <si>
     <t>Keterangan Kalkulasi</t>
   </si>
   <si>
@@ -94,6 +97,15 @@
   </si>
   <si>
     <t>Bon Tambahan+Penerimaan+Antar Teller-Pembayaran-Setor Tambahan-Antar Teller</t>
+  </si>
+  <si>
+    <t>Estim Kredit - (Bon Pagi+Bon Tambahan)+Setor Tambahan-Antar Teller</t>
+  </si>
+  <si>
+    <t>Antar Teller Debet</t>
+  </si>
+  <si>
+    <t>Antar Teller Kredit</t>
   </si>
 </sst>
 </file>
@@ -466,156 +478,155 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{315866AA-0F36-46AA-AD6C-81F0988BC635}">
   <dimension ref="A1:C13"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="14.140625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="16.85546875" customWidth="1"/>
-    <col min="3" max="3" width="75.5703125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="14.1796875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="16.81640625" customWidth="1"/>
+    <col min="3" max="3" width="75.54296875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.35">
       <c r="B1" s="1" t="s">
         <v>0</v>
       </c>
       <c r="C1" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>1</v>
       </c>
       <c r="B2" s="2">
-        <v>5961542438</v>
+        <v>313963390</v>
       </c>
       <c r="C2" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>3</v>
       </c>
       <c r="B3" s="2">
-        <v>6236018261</v>
+        <v>409194311</v>
       </c>
       <c r="C3" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>5</v>
       </c>
       <c r="B4" s="1">
-        <v>310608100</v>
+        <v>86070100</v>
       </c>
       <c r="C4" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
         <v>7</v>
       </c>
       <c r="B5" s="1">
-        <f>4325000000+17000000</f>
-        <v>4342000000</v>
+        <v>0</v>
       </c>
       <c r="C5" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
         <v>9</v>
       </c>
       <c r="B6" s="1">
-        <f>B3-(B4+B5)+B9</f>
-        <v>4323410161</v>
+        <f>B3-(B4+B5)+B9-B7</f>
+        <v>123124211</v>
       </c>
       <c r="C6" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A7" t="s">
+        <v>22</v>
+      </c>
+      <c r="B7" s="1">
+        <v>200000000</v>
+      </c>
+      <c r="C7" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A7" t="s">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A8" t="s">
         <v>10</v>
       </c>
-      <c r="B7" s="1">
-        <v>0</v>
-      </c>
-      <c r="C7" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A8" t="s">
-        <v>11</v>
-      </c>
       <c r="B8" s="1">
-        <f>B2</f>
-        <v>5961542438</v>
+        <f>B2-B10</f>
+        <v>158963390</v>
       </c>
       <c r="C8" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
+        <v>11</v>
+      </c>
+      <c r="B9" s="1">
+        <v>0</v>
+      </c>
+      <c r="C9" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A10" t="s">
+        <v>23</v>
+      </c>
+      <c r="B10" s="1">
+        <v>155000000</v>
+      </c>
+      <c r="C10" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="11" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A11" t="s">
         <v>12</v>
-      </c>
-      <c r="B9" s="1">
-        <v>2740000000</v>
-      </c>
-      <c r="C9" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A10" t="s">
-        <v>10</v>
-      </c>
-      <c r="B10" s="1">
-        <v>0</v>
-      </c>
-      <c r="C10" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A11" t="s">
-        <v>13</v>
       </c>
       <c r="B11" s="1">
         <f>B4+B5+B6+B7-B8-B9-B10</f>
-        <v>274475823</v>
+        <v>95230921</v>
       </c>
       <c r="C11" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="12" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B12" s="2">
-        <v>274475900</v>
+        <v>95231000</v>
       </c>
       <c r="C12" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="13" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A13" s="1" t="s">
         <v>19</v>
-      </c>
-    </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A13" s="1" t="s">
-        <v>21</v>
       </c>
       <c r="B13" s="1">
         <f>B12-B11</f>
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="C13" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
     </row>
   </sheetData>

</xml_diff>